<commit_message>
fix(S14): Fix CSV fixtures with 7 fields and SBI ACH D column
P1: Fix Axis retail and malformed CSV rows that had 7 fields against 6
columns (NEFT CR rows on 15-10, 25-10 and 'Valid row after errors').
Fixed by combining UTR into narration field using hyphen separator.
Regenerated corresponding XLSX fixtures.

P3: Fix SBI fixture ACH D row - moved amount from Credit to Debit column
since ACH D is a debit transaction. Updated all subsequent balances and
the footer totals accordingly:
- Total Debit: 2,46,850.00 (was 2,36,850.00)
- Total Credit: 7,93,500.00 (was 8,03,500.00)
- Closing Balance: 6,46,650.00 (was 6,66,650.00)

Co-authored-by: Raghav <raghavkhanna268@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/banks/synthetic/axis-malformed-synthetic.xlsx
+++ b/tests/fixtures/banks/synthetic/axis-malformed-synthetic.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:F18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -588,18 +588,15 @@
         <v/>
       </c>
       <c r="C15" t="str">
-        <v>Valid row after errors</v>
+        <v>Valid row after errors-SYNTN26296000041</v>
       </c>
       <c r="D15" t="str">
-        <v>SYNTN26296000041</v>
+        <v/>
       </c>
       <c r="E15" t="str">
-        <v/>
+        <v>30,000.00</v>
       </c>
       <c r="F15" t="str">
-        <v>30,000.00</v>
-      </c>
-      <c r="G15" t="str">
         <v>1,85,350.00</v>
       </c>
     </row>
@@ -656,7 +653,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>